<commit_message>
Rev B outputs generated & ignitor current tests added
Rev B outputs generated
Spreadsheet updated with ignitor tests
</commit_message>
<xml_diff>
--- a/Karman Delta Arm/Rocket arming system.xlsx
+++ b/Karman Delta Arm/Rocket arming system.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adria\Documents\GitHub\AltiumGithub\Karman Delta Arm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A013A45-CA1C-4C34-BFF5-C1293A90118D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D508B82F-D9B1-4458-B342-199AEDC7DB41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="29010" windowHeight="15945" tabRatio="783" activeTab="5" xr2:uid="{C397F53C-48EF-47A2-AFE9-4806826F5736}"/>
+    <workbookView xWindow="0" yWindow="1980" windowWidth="21600" windowHeight="12645" tabRatio="783" activeTab="5" xr2:uid="{C397F53C-48EF-47A2-AFE9-4806826F5736}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="609">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1052" uniqueCount="608">
   <si>
     <t>Failure Mode</t>
   </si>
@@ -1925,9 +1925,6 @@
   </si>
   <si>
     <t>Dates</t>
-  </si>
-  <si>
-    <t>Silkscreen pin 1 dots</t>
   </si>
 </sst>
 </file>
@@ -9423,7 +9420,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03095054-2AE4-4924-A1C8-63632743E825}">
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
@@ -9724,10 +9721,10 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>429</v>
+        <v>585</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>551</v>
+        <v>586</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>517</v>
@@ -9735,16 +9732,22 @@
       <c r="D15" s="1" t="s">
         <v>516</v>
       </c>
+      <c r="E15" s="1" t="s">
+        <v>577</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>536</v>
+      </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>585</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>586</v>
+        <v>582</v>
+      </c>
+      <c r="B16" t="s">
+        <v>580</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>517</v>
+        <v>584</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>516</v>
@@ -9758,10 +9761,10 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>582</v>
-      </c>
-      <c r="B17" t="s">
-        <v>580</v>
+        <v>581</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>583</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>584</v>
@@ -9778,10 +9781,10 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>583</v>
+        <v>590</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>584</v>
@@ -9790,7 +9793,7 @@
         <v>516</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>577</v>
+        <v>606</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>536</v>
@@ -9798,10 +9801,10 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>584</v>
@@ -9809,48 +9812,60 @@
       <c r="D19" s="1" t="s">
         <v>516</v>
       </c>
+      <c r="E19" s="1" t="s">
+        <v>593</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>536</v>
+      </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>588</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>589</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>584</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>593</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>536</v>
+        <v>607</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>607</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" t="s">
-        <v>608</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="15">
-      <c r="A25" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15">
+      <c r="A24" s="5" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="42.75">
+    <row r="25" spans="1:7" ht="42.75">
+      <c r="A25" t="s">
+        <v>537</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>517</v>
@@ -9859,15 +9874,15 @@
         <v>516</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>591</v>
+        <v>578</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>517</v>
@@ -9875,16 +9890,13 @@
       <c r="D27" s="1" t="s">
         <v>516</v>
       </c>
-      <c r="G27" s="1" t="s">
-        <v>578</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
+    </row>
+    <row r="28" spans="1:7" ht="57">
       <c r="A28" t="s">
-        <v>542</v>
+        <v>485</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>543</v>
+        <v>548</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>517</v>
@@ -9893,12 +9905,12 @@
         <v>516</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="57">
+    <row r="29" spans="1:7">
       <c r="A29" t="s">
-        <v>485</v>
+        <v>520</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>548</v>
+        <v>521</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>517</v>
@@ -9907,12 +9919,12 @@
         <v>516</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
+    <row r="30" spans="1:7" ht="28.5">
       <c r="A30" t="s">
-        <v>520</v>
+        <v>531</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>521</v>
+        <v>532</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>517</v>
@@ -9920,13 +9932,16 @@
       <c r="D30" s="1" t="s">
         <v>516</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" ht="28.5">
+      <c r="G30" s="1" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
       <c r="A31" t="s">
-        <v>531</v>
+        <v>513</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>532</v>
+        <v>547</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>517</v>
@@ -9935,23 +9950,6 @@
         <v>516</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>595</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="A32" t="s">
-        <v>513</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>517</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>516</v>
-      </c>
-      <c r="G32" s="1" t="s">
         <v>594</v>
       </c>
     </row>

</xml_diff>